<commit_message>
Update soccer trades 2026-08-01 18:02:42 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Premiership/trades.xlsx
+++ b/data/sxbet/ligas/Premiership/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V28"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
+          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>221.54</t>
+          <t>540.4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.4112</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -578,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785603521</t>
+          <t>1785606461</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>538.699088</t>
+          <t>1228.181818</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
+          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,23 +651,31 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>40.12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.515</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -682,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -712,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785603172</t>
+          <t>1785606213</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>77.902913</t>
+          <t>15.503876</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,31 +755,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
+          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>18.89</t>
+          <t>16.26</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4075</t>
+          <t>1.0938</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -786,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -816,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785602480</t>
+          <t>1785606061</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>46.355828</t>
+          <t>173.44</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,31 +867,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
+          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>120.15</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -890,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -920,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785602424</t>
+          <t>1785606042</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -930,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>11.482759</t>
+          <t>218.454545</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,23 +979,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
+          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>113.82262</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.0962</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -971,7 +1007,11 @@
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -994,7 +1034,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1024,7 +1064,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785605997</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1034,7 +1074,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>14.092715</t>
+          <t>1182.572675</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1051,39 +1091,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
+          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>111.28764</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Asian Handicap (1)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1106,7 +1138,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1136,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785604719</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1146,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>48.537549</t>
+          <t>227.117633</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,23 +1195,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
+          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>10.08</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.6025</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1187,7 +1223,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1240,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785600583</t>
+          <t>1785604200</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1250,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>16.73029</t>
+          <t>1.459854</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1267,12 +1307,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
+          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1282,12 +1322,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1297,24 +1337,24 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1322,7 +1362,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1352,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785600448</t>
+          <t>1785604180</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1362,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>30.651341</t>
+          <t>3.591241</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,12 +1419,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
+          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1394,22 +1434,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>7.12</t>
+          <t>20.7</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1434,7 +1474,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1464,7 +1504,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785600138</t>
+          <t>1785604028</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1474,7 +1514,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>22.513834</t>
+          <t>147.857143</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,23 +1531,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
+          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>622.70999</t>
+          <t>58.43</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.1062</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1515,7 +1559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1538,7 +1586,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1568,7 +1616,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785599983</t>
+          <t>1785604011</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1578,7 +1626,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1044.377342</t>
+          <t>549.929412</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1595,12 +1643,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
+          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1610,39 +1658,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1142.73999</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3275</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1650,7 +1698,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1680,7 +1728,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785598284</t>
+          <t>1785604008</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1690,7 +1738,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>3.053435</t>
+          <t>1533.879181</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,12 +1755,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
+          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1722,22 +1770,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>37.20755</t>
+          <t>79.19</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.1387</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Aberdeen +0.5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1762,7 +1810,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1792,7 +1840,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785598183</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1802,7 +1850,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>62.797553</t>
+          <t>570.738739</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,12 +1867,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
+          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1834,22 +1882,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>253.59</t>
+          <t>238.03781</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>Under/Over (3)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Aberdeen +0.5</t>
+          <t>Over 3.0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1874,7 +1922,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1904,7 +1952,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785598181</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1914,7 +1962,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>428.0</t>
+          <t>729.617808</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,28 +1979,28 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
+          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>26.19</t>
+          <t>221.54</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.4112</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Premiership</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1978,7 +2026,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2008,7 +2056,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785597811</t>
+          <t>1785603521</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2018,7 +2066,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>48.165517</t>
+          <t>538.699088</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,67 +2083,59 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
+          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>118.87998</t>
+          <t>40.12</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.9175</t>
+          <t>1.515</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Celtic</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Celtic vs Dundee FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Dundee FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19228045</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2120,17 +2160,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785597330</t>
+          <t>1785603172</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>129.56946</t>
+          <t>77.902913</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2147,7 +2187,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
+          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2158,17 +2198,17 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>18.89</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.4075</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2194,7 +2234,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2224,7 +2264,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785543200</t>
+          <t>1785602480</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2234,7 +2274,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>1.713062</t>
+          <t>46.355828</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2251,28 +2291,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
+          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>40.29346</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -2283,27 +2323,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2328,17 +2368,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785529916</t>
+          <t>1785602424</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>90.293468</t>
+          <t>11.482759</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2355,7 +2395,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
+          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2366,17 +2406,17 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -2387,27 +2427,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2432,17 +2472,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785529915</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2.577031</t>
+          <t>14.092715</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2459,7 +2499,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
+          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2467,23 +2507,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.4175</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2491,27 +2539,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2536,17 +2584,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785529816</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2.754491</t>
+          <t>48.537549</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2563,7 +2611,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
+          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2574,17 +2622,17 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10.08</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.6025</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2595,27 +2643,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2640,17 +2688,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785529105</t>
+          <t>1785600583</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>16.73029</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2667,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
+          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2675,23 +2723,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2699,27 +2755,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2744,17 +2800,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785600448</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>6.77512</t>
+          <t>30.651341</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2771,23 +2827,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
+          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7.12</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2795,7 +2855,11 @@
           <t>Under/Over (3.5)</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2803,27 +2867,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2848,17 +2912,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785600138</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>22.513834</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2875,39 +2939,31 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
+          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>75.44</t>
+          <t>622.70999</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.1313</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2915,27 +2971,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2960,17 +3016,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785599983</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>574.780952</t>
+          <t>1044.377342</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2987,12 +3043,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
+          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3002,22 +3058,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>169.77</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.3275</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -3027,27 +3083,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3072,17 +3128,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785598284</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1061.0625</t>
+          <t>3.053435</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3099,7 +3155,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3107,23 +3163,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>20.18</t>
+          <t>37.20755</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3887</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Aberdeen +0.5</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3131,27 +3195,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3176,17 +3240,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785526560</t>
+          <t>1785598183</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>51.909968</t>
+          <t>62.797553</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3203,12 +3267,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3218,22 +3282,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>61.03</t>
+          <t>253.59</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.0925</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>Asian Handicap (0.5)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Over 5.0</t>
+          <t>Aberdeen +0.5</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3243,27 +3307,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3288,17 +3352,17 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785524635</t>
+          <t>1785598181</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>659.783784</t>
+          <t>428.0</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3315,110 +3379,1494 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>26.19</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.5437</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19228039</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1785597811</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1785601800</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>48.165517</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>118.87998</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.9175</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Celtic vs Dundee FC</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Dundee FC</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19228045</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1785597330</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1785781800</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>129.56946</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.5837</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19228039</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1785543200</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1785601800</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>1.713062</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>40.29346</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.4463</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1785529916</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>90.293468</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.4463</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1785529915</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2.577031</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.4175</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1785529816</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>2.754491</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1785529105</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>1.587302</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.2612</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1785529104</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>6.77512</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1785529104</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>1.587302</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>75.44</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.1313</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Over 4.5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1785526843</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>574.780952</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>169.77</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1785526843</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>1061.0625</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>20.18</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.3887</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1785526560</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>51.909968</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>61.03</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.0925</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1785524635</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>659.783784</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>0x3a6afc0d74597a50f894e10c8d93084fcb7ca5e09aa24a3eab1b5f521c2b6e08</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>0xCCdf6F3306aa9df4a4852FaF67fA1e1D58c4Db4e</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>176.04</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>1.495</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Under/Over (3)</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>Over 3.0</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>Dundee United vs Rangers FC</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Dundee United</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>Rangers FC</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>0x2af09a7c30a9c2f3a49f480d1eba3b8573b203b8cb5cec998c89bf8da583850a</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>L19228047</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
         <is>
           <t>1785524138</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="S41" t="inlineStr">
         <is>
           <t>1785524400</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="T41" t="inlineStr">
         <is>
           <t>355.636364</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V28" t="inlineStr">
+      <c r="V41" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-02 01:02:36 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Premiership/trades.xlsx
+++ b/data/sxbet/ligas/Premiership/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x119739feb921ac6aaf1c73d753c84fe8b4ef7a1d89b8d653c384bcb65d17eb44</t>
+          <t>0x6ab196073a2c34a857b463177bac529748ff13ee57f0aec52e6f6fc643ae0718</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,23 +539,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7225</t>
+          <t>1.485</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>St. Johnstone vs Kilmarnock</t>
+          <t>Hibernian vs Motherwell</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>St. Johnstone</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Kilmarnock</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x23b587c4d4eadaf253c4b86c75fcdd4ec70729ea8567febc472ad12253b9fe16</t>
+          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19228040</t>
+          <t>L19228046</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785623149</t>
+          <t>1785630118</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785675600</t>
+          <t>1785684600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>3.847751</t>
+          <t>7.175258</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,39 +643,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
+          <t>0x119739feb921ac6aaf1c73d753c84fe8b4ef7a1d89b8d653c384bcb65d17eb44</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>540.4</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.7225</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x23b587c4d4eadaf253c4b86c75fcdd4ec70729ea8567febc472ad12253b9fe16</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785606461</t>
+          <t>1785623149</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1228.181818</t>
+          <t>3.847751</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
+          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,22 +762,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>540.4</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785606213</t>
+          <t>1785606461</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>15.503876</t>
+          <t>1228.181818</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
+          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,39 +874,39 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16.26</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.0938</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -914,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785606061</t>
+          <t>1785606213</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>173.44</t>
+          <t>15.503876</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
+          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,22 +986,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>120.15</t>
+          <t>16.26</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.0938</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785606042</t>
+          <t>1785606061</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>218.454545</t>
+          <t>173.44</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
+          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1098,39 +1098,39 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>113.82262</t>
+          <t>120.15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.0962</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785605997</t>
+          <t>1785606042</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1182.572675</t>
+          <t>218.454545</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1195,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
+          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1203,23 +1203,31 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>111.28764</t>
+          <t>113.82262</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.0962</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1242,7 +1250,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1272,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785604719</t>
+          <t>1785605997</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>227.117633</t>
+          <t>1182.572675</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,62 +1307,54 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
+          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>111.28764</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
+          <t>Asian Handicap (1)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Heart of Midlothian</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785604200</t>
+          <t>1785604719</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.459854</t>
+          <t>227.117633</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,12 +1411,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
+          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
+          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785604180</t>
+          <t>1785604200</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>3.591241</t>
+          <t>1.459854</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,12 +1523,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
+          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1538,39 +1538,39 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785604028</t>
+          <t>1785604180</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>147.857143</t>
+          <t>3.591241</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,7 +1635,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
+          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1650,17 +1650,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>58.43</t>
+          <t>20.7</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.1062</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1720,7 +1720,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785604011</t>
+          <t>1785604028</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>549.929412</t>
+          <t>147.857143</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1747,7 +1747,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
+          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1762,22 +1762,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1142.73999</t>
+          <t>58.43</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.1062</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785604008</t>
+          <t>1785604011</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>1533.879181</t>
+          <t>549.929412</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1859,7 +1859,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
+          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1874,39 +1874,39 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>79.19</t>
+          <t>1142.73999</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.1387</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785604004</t>
+          <t>1785604008</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>570.738739</t>
+          <t>1533.879181</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
+          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1986,22 +1986,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>238.03781</t>
+          <t>79.19</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.1387</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>729.617808</t>
+          <t>570.738739</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2083,31 +2083,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
+          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>221.54</t>
+          <t>238.03781</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.4112</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2130,7 +2138,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2160,7 +2168,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785603521</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2170,7 +2178,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>538.699088</t>
+          <t>729.617808</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2187,28 +2195,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
+          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>40.12</t>
+          <t>221.54</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.515</t>
+          <t>1.4112</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2234,7 +2242,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2264,7 +2272,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785603172</t>
+          <t>1785603521</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2274,7 +2282,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>77.902913</t>
+          <t>538.699088</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2291,23 +2299,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
+          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>18.89</t>
+          <t>40.12</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4075</t>
+          <t>1.515</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2368,7 +2376,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785602480</t>
+          <t>1785603172</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2378,7 +2386,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>46.355828</t>
+          <t>77.902913</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2395,7 +2403,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
+          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2406,17 +2414,17 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>18.89</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.4075</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -2442,7 +2450,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2472,7 +2480,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785602424</t>
+          <t>1785602480</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2482,7 +2490,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>11.482759</t>
+          <t>46.355828</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,7 +2507,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
+          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2510,17 +2518,17 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Premiership</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -2546,7 +2554,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2576,7 +2584,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785602424</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2586,7 +2594,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>14.092715</t>
+          <t>11.482759</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2603,7 +2611,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
+          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2611,31 +2619,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>48.537549</t>
+          <t>14.092715</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2715,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
+          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2723,23 +2723,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10.08</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.6025</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2762,7 +2770,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2792,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785600583</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2802,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>16.73029</t>
+          <t>48.537549</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2819,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
+          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2827,19 +2835,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>10.08</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.6025</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2847,26 +2851,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K23" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785600448</t>
+          <t>1785600583</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>30.651341</t>
+          <t>16.73029</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,12 +2931,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
+          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2946,22 +2946,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>7.12</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785600138</t>
+          <t>1785600448</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>22.513834</t>
+          <t>30.651341</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3043,7 +3043,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
+          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3051,23 +3051,31 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>622.70999</t>
+          <t>7.12</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3090,7 +3098,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3120,7 +3128,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785599983</t>
+          <t>1785600138</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3130,7 +3138,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>1044.377342</t>
+          <t>22.513834</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3147,27 +3155,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
+          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>622.70999</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3275</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3175,26 +3179,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785598284</t>
+          <t>1785599983</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>3.053435</t>
+          <t>1044.377342</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3259,12 +3259,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
+          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3274,22 +3274,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>37.20755</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.3275</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Aberdeen +0.5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785598183</t>
+          <t>1785598284</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>62.797553</t>
+          <t>3.053435</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3371,7 +3371,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
+          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>253.59</t>
+          <t>37.20755</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785598181</t>
+          <t>1785598183</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>428.0</t>
+          <t>62.797553</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3483,36 +3483,44 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
+          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>26.19</t>
+          <t>253.59</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Aberdeen +0.5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>Aberdeen vs Heart of Midlothian</t>
@@ -3530,7 +3538,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3560,7 +3568,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785597811</t>
+          <t>1785598181</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3570,7 +3578,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>48.165517</t>
+          <t>428.0</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3587,27 +3595,23 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
+          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>118.87998</t>
+          <t>26.19</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.9175</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3615,11 +3619,7 @@
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Celtic</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3627,27 +3627,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Celtic vs Dundee FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Dundee FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19228045</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3672,17 +3672,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785597330</t>
+          <t>1785597811</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>129.56946</t>
+          <t>48.165517</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,31 +3699,39 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
+          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>118.87998</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.9175</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3731,27 +3739,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>Celtic vs Dundee FC</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Dundee FC</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228045</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3776,17 +3784,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785543200</t>
+          <t>1785597330</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>1.713062</t>
+          <t>129.56946</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3803,28 +3811,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
+          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>40.29346</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -3835,27 +3843,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3880,17 +3888,17 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785529916</t>
+          <t>1785543200</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>90.293468</t>
+          <t>1.713062</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3907,18 +3915,18 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
+          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>40.29346</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3984,7 +3992,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785529915</t>
+          <t>1785529916</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3994,7 +4002,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>2.577031</t>
+          <t>90.293468</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4011,7 +4019,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
+          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4027,7 +4035,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.4175</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4088,7 +4096,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785529816</t>
+          <t>1785529915</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4098,7 +4106,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2.754491</t>
+          <t>2.577031</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4115,7 +4123,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
+          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4126,17 +4134,17 @@
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.4175</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -4162,7 +4170,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4192,7 +4200,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785529105</t>
+          <t>1785529816</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4202,7 +4210,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>2.754491</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4219,7 +4227,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
+          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4230,17 +4238,17 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -4266,7 +4274,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4296,7 +4304,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785529105</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4306,7 +4314,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>6.77512</t>
+          <t>1.587302</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4323,7 +4331,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
+          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4334,17 +4342,17 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -4370,7 +4378,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4410,7 +4418,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>6.77512</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4427,39 +4435,31 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
+          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>75.44</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.1313</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785529104</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>574.780952</t>
+          <t>1.587302</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4539,7 +4539,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
+          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4554,22 +4554,22 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>169.77</t>
+          <t>75.44</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.1313</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
+          <t>Under/Over (4.5)</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Over 4.0</t>
+          <t>Over 4.5</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
+          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>1061.0625</t>
+          <t>574.780952</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4651,31 +4651,39 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>20.18</t>
+          <t>169.77</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.3887</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4698,7 +4706,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4728,7 +4736,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785526560</t>
+          <t>1785526843</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4738,7 +4746,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>51.909968</t>
+          <t>1061.0625</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4755,39 +4763,31 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>61.03</t>
+          <t>20.18</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.0925</t>
+          <t>1.3887</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4810,7 +4810,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785524635</t>
+          <t>1785526560</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>659.783784</t>
+          <t>51.909968</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4867,110 +4867,222 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>61.03</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.0925</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1785524635</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>659.783784</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>0x3a6afc0d74597a50f894e10c8d93084fcb7ca5e09aa24a3eab1b5f521c2b6e08</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>0xCCdf6F3306aa9df4a4852FaF67fA1e1D58c4Db4e</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>176.04</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>1.495</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Under/Over (3)</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Over 3.0</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>Dundee United vs Rangers FC</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Dundee United</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>Rangers FC</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>0x2af09a7c30a9c2f3a49f480d1eba3b8573b203b8cb5cec998c89bf8da583850a</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>L19228047</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
         <is>
           <t>1785524138</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr">
+      <c r="S43" t="inlineStr">
         <is>
           <t>1785524400</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T43" t="inlineStr">
         <is>
           <t>355.636364</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V43" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-02 03:02:52 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Premiership/trades.xlsx
+++ b/data/sxbet/ligas/Premiership/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V43"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x6ab196073a2c34a857b463177bac529748ff13ee57f0aec52e6f6fc643ae0718</t>
+          <t>0x75ef518b65fe522ded9c78a1d5f31a90d2901382f170023f7b6dd2d74fefc9ff</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -539,31 +539,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.485</t>
+          <t>1.635</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -571,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Hibernian vs Motherwell</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Hibernian</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Motherwell</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
+          <t>0x53a71c3f6c6ea99c0a39f725804b4ea70d4a29654a2903d942ccfb92e2bcd5c3</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19228046</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785630118</t>
+          <t>1785636203</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785684600</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>7.175258</t>
+          <t>1.574803</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x119739feb921ac6aaf1c73d753c84fe8b4ef7a1d89b8d653c384bcb65d17eb44</t>
+          <t>0x828cc7a1897c5fc5bc4301f9a7440aeda6cda8fac90ae0bd1c98ee5719a0f76e</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -651,23 +643,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7225</t>
+          <t>1.4912</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>St. Johnstone vs Kilmarnock</t>
+          <t>Hibernian vs Motherwell</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>St. Johnstone</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Kilmarnock</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x23b587c4d4eadaf253c4b86c75fcdd4ec70729ea8567febc472ad12253b9fe16</t>
+          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19228040</t>
+          <t>L19228046</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785623149</t>
+          <t>1785635973</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785675600</t>
+          <t>1785684600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>3.847751</t>
+          <t>20.356234</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
+          <t>0x6ab196073a2c34a857b463177bac529748ff13ee57f0aec52e6f6fc643ae0718</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,22 +762,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>540.4</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.485</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -787,27 +787,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>Hibernian vs Motherwell</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228046</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +832,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785606461</t>
+          <t>1785630118</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785684600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>1228.181818</t>
+          <t>7.175258</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,39 +859,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
+          <t>0x119739feb921ac6aaf1c73d753c84fe8b4ef7a1d89b8d653c384bcb65d17eb44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.7225</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
+          <t>0x23b587c4d4eadaf253c4b86c75fcdd4ec70729ea8567febc472ad12253b9fe16</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785606213</t>
+          <t>1785623149</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>15.503876</t>
+          <t>3.847751</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
+          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,39 +978,39 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>16.26</t>
+          <t>540.4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.0938</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1026,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785606061</t>
+          <t>1785606461</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>173.44</t>
+          <t>1228.181818</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1075,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
+          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>120.15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1138,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1168,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785606042</t>
+          <t>1785606213</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1178,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>218.454545</t>
+          <t>15.503876</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,7 +1187,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
+          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1210,12 +1202,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>113.82262</t>
+          <t>16.26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.0962</t>
+          <t>1.0938</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1280,7 +1272,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785605997</t>
+          <t>1785606061</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1290,7 +1282,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1182.572675</t>
+          <t>173.44</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1307,7 +1299,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
+          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1315,23 +1307,31 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>111.28764</t>
+          <t>120.15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785604719</t>
+          <t>1785606042</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>227.117633</t>
+          <t>218.454545</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,12 +1411,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
+          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1426,47 +1426,47 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>113.82262</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.0962</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>Heart of Midlothian</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Heart of Midlothian</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785604200</t>
+          <t>1785605997</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1.459854</t>
+          <t>1182.572675</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,62 +1523,54 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
+          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>111.28764</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
+          <t>Asian Handicap (1)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Heart of Midlothian</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1608,7 +1600,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785604180</t>
+          <t>1785604719</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1618,7 +1610,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>3.591241</t>
+          <t>227.117633</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1635,12 +1627,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
+          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1650,39 +1642,39 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1690,7 +1682,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1720,7 +1712,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785604028</t>
+          <t>1785604200</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1730,7 +1722,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>147.857143</t>
+          <t>1.459854</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1747,12 +1739,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
+          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1762,12 +1754,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>58.43</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.1062</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1777,24 +1769,24 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1802,7 +1794,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1832,7 +1824,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785604011</t>
+          <t>1785604180</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1842,7 +1834,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>549.929412</t>
+          <t>3.591241</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1859,7 +1851,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
+          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1874,22 +1866,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1142.73999</t>
+          <t>20.7</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1914,7 +1906,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1944,7 +1936,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785604008</t>
+          <t>1785604028</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1954,7 +1946,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1533.879181</t>
+          <t>147.857143</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1971,7 +1963,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
+          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1986,39 +1978,39 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>79.19</t>
+          <t>58.43</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.1387</t>
+          <t>1.1062</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -2026,7 +2018,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2056,7 +2048,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785604004</t>
+          <t>1785604011</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2066,7 +2058,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>570.738739</t>
+          <t>549.929412</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2083,7 +2075,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
+          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2098,22 +2090,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>238.03781</t>
+          <t>1142.73999</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2138,7 +2130,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2168,7 +2160,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785604004</t>
+          <t>1785604008</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2178,7 +2170,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>729.617808</t>
+          <t>1533.879181</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2195,31 +2187,39 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
+          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>221.54</t>
+          <t>79.19</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.4112</t>
+          <t>1.1387</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785603521</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>538.699088</t>
+          <t>570.738739</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2299,31 +2299,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
+          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>40.12</t>
+          <t>238.03781</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.515</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2346,7 +2354,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2376,7 +2384,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785603172</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2386,7 +2394,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>77.902913</t>
+          <t>729.617808</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2403,7 +2411,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
+          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2414,17 +2422,17 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>18.89</t>
+          <t>221.54</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4075</t>
+          <t>1.4112</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -2450,7 +2458,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2480,7 +2488,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785602480</t>
+          <t>1785603521</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2490,7 +2498,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>46.355828</t>
+          <t>538.699088</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2507,28 +2515,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
+          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>40.12</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.515</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -2554,7 +2562,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2584,7 +2592,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785602424</t>
+          <t>1785603172</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2594,7 +2602,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>11.482759</t>
+          <t>77.902913</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2611,7 +2619,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
+          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2622,17 +2630,17 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>18.89</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.4075</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Premiership</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2658,7 +2666,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2688,7 +2696,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785602480</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2698,7 +2706,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>14.092715</t>
+          <t>46.355828</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2715,7 +2723,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
+          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2723,31 +2731,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2770,7 +2770,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785602424</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>48.537549</t>
+          <t>11.482759</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
+          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2838,17 +2838,17 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10.08</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.6025</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785600583</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>16.73029</t>
+          <t>14.092715</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,7 +2931,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
+          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2946,39 +2946,39 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3016,7 +3016,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785600448</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>30.651341</t>
+          <t>48.537549</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3043,39 +3043,31 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
+          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>7.12</t>
+          <t>10.08</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.6025</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3098,7 +3090,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3128,7 +3120,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785600138</t>
+          <t>1785600583</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3138,7 +3130,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>22.513834</t>
+          <t>16.73029</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3155,23 +3147,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
+          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>622.70999</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3179,7 +3175,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785599983</t>
+          <t>1785600448</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>1044.377342</t>
+          <t>30.651341</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3259,12 +3259,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
+          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3274,39 +3274,39 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7.12</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3275</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785598284</t>
+          <t>1785600138</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>3.053435</t>
+          <t>22.513834</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3371,39 +3371,31 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
+          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>37.20755</t>
+          <t>622.70999</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Aberdeen +0.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3426,7 +3418,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3456,7 +3448,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785598183</t>
+          <t>1785599983</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3466,7 +3458,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>62.797553</t>
+          <t>1044.377342</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3483,12 +3475,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
+          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3498,22 +3490,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>253.59</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.3275</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Aberdeen +0.5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -3538,7 +3530,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3568,7 +3560,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785598181</t>
+          <t>1785598284</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3578,7 +3570,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>428.0</t>
+          <t>3.053435</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3595,36 +3587,44 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
+          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>26.19</t>
+          <t>37.20755</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Aberdeen +0.5</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>Aberdeen vs Heart of Midlothian</t>
@@ -3642,7 +3642,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785597811</t>
+          <t>1785598183</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>48.165517</t>
+          <t>62.797553</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,12 +3699,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
+          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3714,52 +3714,52 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>118.87998</t>
+          <t>253.59</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.9175</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Aberdeen +0.5</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Celtic</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Celtic vs Dundee FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Dundee FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19228045</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3784,17 +3784,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785597330</t>
+          <t>1785598181</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>129.56946</t>
+          <t>428.0</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3811,28 +3811,28 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
+          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>26.19</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785543200</t>
+          <t>1785597811</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1.713062</t>
+          <t>48.165517</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,31 +3915,39 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
+          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>40.29346</t>
+          <t>118.87998</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.9175</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3947,27 +3955,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Celtic vs Dundee FC</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Dundee FC</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228045</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3992,17 +4000,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785529916</t>
+          <t>1785597330</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>90.293468</t>
+          <t>129.56946</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4019,7 +4027,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
+          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4030,17 +4038,17 @@
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -4051,27 +4059,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4096,17 +4104,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785529915</t>
+          <t>1785543200</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>2.577031</t>
+          <t>1.713062</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4123,23 +4131,23 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
+          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>40.29346</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.4175</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4200,7 +4208,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785529816</t>
+          <t>1785529916</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4210,7 +4218,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>2.754491</t>
+          <t>90.293468</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4227,7 +4235,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
+          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4238,17 +4246,17 @@
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -4274,7 +4282,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4304,7 +4312,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785529105</t>
+          <t>1785529915</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4314,7 +4322,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>2.577031</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4331,7 +4339,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
+          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4342,12 +4350,12 @@
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.4175</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -4408,7 +4416,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785529816</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4418,7 +4426,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>6.77512</t>
+          <t>2.754491</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4435,7 +4443,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
+          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4512,7 +4520,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785529105</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4539,39 +4547,31 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
+          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>75.44</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.1313</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -4624,7 +4624,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785529104</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>574.780952</t>
+          <t>6.77512</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4651,39 +4651,31 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
+          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>169.77</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Over 4.0</t>
-        </is>
-      </c>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4706,7 +4698,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4736,7 +4728,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785529104</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4746,7 +4738,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1061.0625</t>
+          <t>1.587302</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4763,31 +4755,39 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>20.18</t>
+          <t>75.44</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.3887</t>
+          <t>1.1313</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Over 4.5</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4810,7 +4810,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4840,7 +4840,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785526560</t>
+          <t>1785526843</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4850,7 +4850,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>51.909968</t>
+          <t>574.780952</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4867,7 +4867,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4882,22 +4882,22 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>61.03</t>
+          <t>169.77</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.0925</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
+          <t>Under/Over (4)</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Over 5.0</t>
+          <t>Over 4.0</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785524635</t>
+          <t>1785526843</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>659.783784</t>
+          <t>1061.0625</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4979,110 +4979,326 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>20.18</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.3887</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1785526560</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>51.909968</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>61.03</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.0925</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1785524635</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>659.783784</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>0x3a6afc0d74597a50f894e10c8d93084fcb7ca5e09aa24a3eab1b5f521c2b6e08</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>0xCCdf6F3306aa9df4a4852FaF67fA1e1D58c4Db4e</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
         <is>
           <t>176.04</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>1.495</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Under/Over (3)</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>Over 3.0</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Dundee United vs Rangers FC</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J45" t="inlineStr">
         <is>
           <t>Dundee United</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Rangers FC</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>0x2af09a7c30a9c2f3a49f480d1eba3b8573b203b8cb5cec998c89bf8da583850a</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>L19228047</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
         <is>
           <t>1785524138</t>
         </is>
       </c>
-      <c r="S43" t="inlineStr">
+      <c r="S45" t="inlineStr">
         <is>
           <t>1785524400</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="T45" t="inlineStr">
         <is>
           <t>355.636364</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="U45" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
+      <c r="V45" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-02 10:02:27 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Premiership/trades.xlsx
+++ b/data/sxbet/ligas/Premiership/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V45"/>
+  <dimension ref="A1:V50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x75ef518b65fe522ded9c78a1d5f31a90d2901382f170023f7b6dd2d74fefc9ff</t>
+          <t>0xa3246839c82e1d3b7b79ec7134f5e16ac34c978224c73f9cf936402bb3f46246</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x3c0287d63932634992dC40382ee8C4Fa83681Dd1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>22.47</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.635</t>
+          <t>1.4387</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Hibernian</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>St. Johnstone vs Kilmarnock</t>
+          <t>Hibernian vs Motherwell</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>St. Johnstone</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Kilmarnock</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x53a71c3f6c6ea99c0a39f725804b4ea70d4a29654a2903d942ccfb92e2bcd5c3</t>
+          <t>0x9f1a3561e16a2d0b3c37f6e3c72434f322dfbe1a4e4f2db43c4834fec7e37ca8</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19228040</t>
+          <t>L19228046</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1785636203</t>
+          <t>1785662110</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1785675600</t>
+          <t>1785684600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1.574803</t>
+          <t>51.213675</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x828cc7a1897c5fc5bc4301f9a7440aeda6cda8fac90ae0bd1c98ee5719a0f76e</t>
+          <t>0x1d1e098954f1c91c97a06acd702caf64f5c976927b5cfeaca5e2eb798a33b4e4</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,31 +651,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>39.80897</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.4912</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Hibernian vs Motherwell</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Hibernian</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Motherwell</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
+          <t>0xbebf21a64fc9e69fed2003bb3aaf7e9db7162dbf82e179c3e21769683becd2a1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19228046</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1785635973</t>
+          <t>1785660888</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1785684600</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>20.356234</t>
+          <t>56.068972</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,12 +747,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x6ab196073a2c34a857b463177bac529748ff13ee57f0aec52e6f6fc643ae0718</t>
+          <t>0x3a91b4ee4ebe4a44ecdf84e9d6ea4e3c65ba8af4f7422c11d076afba8bf5a45e</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x23a63d3fEDf22e3D422073b7226922d61587207c</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -762,22 +762,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.485</t>
+          <t>1.4387</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
+          <t>0x9f1a3561e16a2d0b3c37f6e3c72434f322dfbe1a4e4f2db43c4834fec7e37ca8</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1785630118</t>
+          <t>1785659879</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>7.175258</t>
+          <t>4.672365</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x119739feb921ac6aaf1c73d753c84fe8b4ef7a1d89b8d653c384bcb65d17eb44</t>
+          <t>0xd47a15b073a363789220e1cf024b7af5305a66f3777fd0039ee12d3de57bd0bf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -870,17 +870,17 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>4.73</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.7225</t>
+          <t>1.4287</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -906,7 +906,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x23b587c4d4eadaf253c4b86c75fcdd4ec70729ea8567febc472ad12253b9fe16</t>
+          <t>0x36bed9ba7cf9a4329b968ce6013308ee218af06f4b67ca9e7013eca5c9631d79</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1785623149</t>
+          <t>1785656458</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>3.847751</t>
+          <t>11.03207</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,39 +963,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
+          <t>0x941e76d7a6a1b26012f4ee31714ecadb8a2a95b32d0be17fbc02b0a5582a1d62</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>540.4</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.4287</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1003,27 +995,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x36bed9ba7cf9a4329b968ce6013308ee218af06f4b67ca9e7013eca5c9631d79</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1040,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1785606461</t>
+          <t>1785656419</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1228.181818</t>
+          <t>2.425656</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,39 +1067,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
+          <t>0x75ef518b65fe522ded9c78a1d5f31a90d2901382f170023f7b6dd2d74fefc9ff</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.3225</t>
+          <t>1.635</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1115,27 +1099,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
+          <t>0x53a71c3f6c6ea99c0a39f725804b4ea70d4a29654a2903d942ccfb92e2bcd5c3</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1144,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1785606213</t>
+          <t>1785636203</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>15.503876</t>
+          <t>1.574803</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,12 +1171,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
+          <t>0x828cc7a1897c5fc5bc4301f9a7440aeda6cda8fac90ae0bd1c98ee5719a0f76e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1202,52 +1186,52 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>16.26</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.0938</t>
+          <t>1.4912</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>Hibernian vs Motherwell</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228046</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1272,17 +1256,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1785606061</t>
+          <t>1785635973</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785684600</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>173.44</t>
+          <t>20.356234</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,12 +1283,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
+          <t>0x6ab196073a2c34a857b463177bac529748ff13ee57f0aec52e6f6fc643ae0718</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1314,22 +1298,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>120.15</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.485</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1339,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>Hibernian vs Motherwell</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x2783261fcb8854d285b611657288b8d77bcc8e0dfdcc94b3e12d815b0c6f0ad1</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228046</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1384,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1785606042</t>
+          <t>1785630118</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785684600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>218.454545</t>
+          <t>7.175258</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,67 +1395,59 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
+          <t>0x119739feb921ac6aaf1c73d753c84fe8b4ef7a1d89b8d653c384bcb65d17eb44</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>113.82262</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.0962</t>
+          <t>1.7225</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
+          <t>St. Johnstone vs Kilmarnock</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Heart of Midlothian</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x23b587c4d4eadaf253c4b86c75fcdd4ec70729ea8567febc472ad12253b9fe16</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19228039</t>
+          <t>L19228040</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1496,17 +1472,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1785605997</t>
+          <t>1785623149</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1785601800</t>
+          <t>1785675600</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>1182.572675</t>
+          <t>3.847751</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1523,7 +1499,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
+          <t>0x285a5fd104f5d7656de510897faa7bd4458d7a455cf677dfe51254fe7ba4d2b6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1531,23 +1507,31 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>111.28764</t>
+          <t>540.4</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Asian Handicap (1)</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -1570,7 +1554,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1600,7 +1584,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1785604719</t>
+          <t>1785606461</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1610,7 +1594,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>227.117633</t>
+          <t>1228.181818</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,12 +1611,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
+          <t>0xf22ffe2952c7c68f8dfc9f2d67c7abc2524fa132087e243d33ec3a6cc341bd65</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1642,47 +1626,47 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.3225</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>Heart of Midlothian</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Heart of Midlothian</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0xe60c02a40f6d793a7b64339680c7a119b47f886321c3addc85f497e35e0ca793</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1696,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1785604200</t>
+          <t>1785606213</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1706,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>1.459854</t>
+          <t>15.503876</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,12 +1723,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
+          <t>0x59fde39b6f148fd1215b657887ed4f43e9a2db36d1798dda0c37e8dfc7fbde76</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1754,47 +1738,47 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>16.26</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.685</t>
+          <t>1.0938</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t>Heart of Midlothian</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Heart of Midlothian</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1785604180</t>
+          <t>1785606061</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>3.591241</t>
+          <t>173.44</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,7 +1835,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
+          <t>0x0e430f6a34ae833d3b326cdb6db44835894df5a80a68df992f04a51a1fbcede8</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1866,39 +1850,39 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>20.7</t>
+          <t>120.15</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -1906,7 +1890,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1936,7 +1920,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1785604028</t>
+          <t>1785606042</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1946,7 +1930,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>147.857143</t>
+          <t>218.454545</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1963,7 +1947,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
+          <t>0xe2f524ccfb2b8ea547b7f17ddfbd89a1865cfb986eb6bc2ce1ce4630f8388d54</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1978,17 +1962,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>58.43</t>
+          <t>113.82262</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.1062</t>
+          <t>1.0962</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2018,7 +2002,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2048,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1785604011</t>
+          <t>1785605997</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2058,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>549.929412</t>
+          <t>1182.572675</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2075,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
+          <t>0x798a2dd92705725f7e43da661a6058835f408eb6bcf6cdf2ebadab6d345eb3a1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2083,31 +2067,23 @@
           <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1142.73999</t>
+          <t>111.28764</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.745</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>Asian Handicap (1)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2130,7 +2106,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x28b154cd868e90e22afd88e0b88b37d60f306ff33bf341cfb50e3c409aac81a7</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2160,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1785604008</t>
+          <t>1785604719</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2170,7 +2146,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>1533.879181</t>
+          <t>227.117633</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2187,12 +2163,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
+          <t>0x848d8d806be9a756592c44678cf4f627ba77b9010fc492c9e3dd32942dc0bff2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0x07708a791d2c7549244E6c62A14B12b09FAAE65D</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2202,39 +2178,39 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>79.19</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.1387</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -2242,7 +2218,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2272,7 +2248,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1785604004</t>
+          <t>1785604200</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2282,7 +2258,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>570.738739</t>
+          <t>1.459854</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2299,12 +2275,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
+          <t>0x925930e535ba2a3cd4d63099999c84a9977750e4607d4f1e3b8f69af1a5bae17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+          <t>0xAB03DDB118c18F7EfC711f056a7A4B5D25e040aA</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2314,22 +2290,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>238.03781</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.685</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (3)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Over 3.0</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2354,7 +2330,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2384,7 +2360,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1785604004</t>
+          <t>1785604180</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2394,7 +2370,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>729.617808</t>
+          <t>3.591241</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2411,31 +2387,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
+          <t>0x4c6a1fd994bbc9b3204ba07f5a25d6d9b2fadcb5868fde25397da4c34af10eec</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>221.54</t>
+          <t>20.7</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.4112</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2458,7 +2442,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2488,7 +2472,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1785603521</t>
+          <t>1785604028</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2498,7 +2482,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>538.699088</t>
+          <t>147.857143</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2515,31 +2499,39 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
+          <t>0x4840850d5a78e921d1d523868aea7485202701a718ec2e7aa0c19b9b4dc54a39</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>40.12</t>
+          <t>58.43</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.515</t>
+          <t>1.1062</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2562,7 +2554,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2592,7 +2584,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1785603172</t>
+          <t>1785604011</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2602,7 +2594,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>77.902913</t>
+          <t>549.929412</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2619,23 +2611,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
+          <t>0xcf645932fc9fc44dcce78623fe36e0b5a2a770c7768c166ded87f80ea4629ad0</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>18.89</t>
+          <t>1142.73999</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.4075</t>
+          <t>1.745</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2643,7 +2639,11 @@
           <t>Under/Over (2)</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1785602480</t>
+          <t>1785604008</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>46.355828</t>
+          <t>1533.879181</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2723,31 +2723,39 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
+          <t>0xee92ca9c29ea82990989cd8f4f18a9271dfaee1ee58ee39ff9d4ea8cae6162fa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>79.19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.1387</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2770,7 +2778,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
+          <t>0x13afa08855879d0fb10ba39752b59dd3851c9a86db3e7d49dcd53265c0a094b8</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2800,7 +2808,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1785602424</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2810,7 +2818,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>11.482759</t>
+          <t>570.738739</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2827,36 +2835,44 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
+          <t>0x481f2136c4218797be6f5498911a758cd98b7d2b25a64fc22ad7599ea294c18f</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>238.03781</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.5663</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
+          <t>Under/Over (3)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Over 3.0</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>Aberdeen vs Heart of Midlothian</t>
@@ -2874,7 +2890,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0xc827c4361285ff3730f2a2827cfaf4c676a98131c5260897f68817741137c35d</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2904,7 +2920,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785604004</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2914,7 +2930,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>14.092715</t>
+          <t>729.617808</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2931,7 +2947,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
+          <t>0xf1ff5187b59c2c170177f0b5168e643e683b6267c1d47d6354dd0c2cd7e3db7f</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2939,31 +2955,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>221.54</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.4112</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -2986,7 +2994,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3016,7 +3024,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1785600627</t>
+          <t>1785603521</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3026,7 +3034,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>48.537549</t>
+          <t>538.699088</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3043,28 +3051,28 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
+          <t>0x7038e38303a9c1caaff6ad103dd90e763a7ed2daf0187c1c30eaf28493a7c535</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10.08</t>
+          <t>40.12</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.6025</t>
+          <t>1.515</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -3090,7 +3098,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3120,7 +3128,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1785600583</t>
+          <t>1785603172</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3130,7 +3138,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>16.73029</t>
+          <t>77.902913</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3147,7 +3155,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
+          <t>0x5593ee9dbf8234ebc5cd2d7f63a0cab2a7089790a5725d69d2bea597242e072a</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3155,46 +3163,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18.89</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.3262</t>
+          <t>1.4075</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K26" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x348e726f6237441e04fb457f50aef2158e209f96c9abe9cde51d535052b0a0ef</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1785600448</t>
+          <t>1785602480</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>30.651341</t>
+          <t>46.355828</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3259,39 +3259,31 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
+          <t>0xdeb734fd55693d6bb57dd13b4a021a04041a2a7e576b65b08d43832ab4f5a527</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>7.12</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.3162</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3314,7 +3306,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
+          <t>0x9a443e546e77e9f80d33b52f010c5e5cb8a79df43a9ca840a543143b3d478ef4</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3344,7 +3336,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1785600138</t>
+          <t>1785602424</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3354,7 +3346,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>22.513834</t>
+          <t>11.482759</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3371,28 +3363,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
+          <t>0xfb04bbcdc9241892746a7738b4d43299feeb4ae5ea1ac018cc8b4cf8c1ce3ed8</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>622.70999</t>
+          <t>7.98</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.5962</t>
+          <t>1.5663</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -3418,7 +3410,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3448,7 +3440,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1785599983</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3458,7 +3450,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>1044.377342</t>
+          <t>14.092715</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3475,12 +3467,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
+          <t>0xd634bf9e90e95d19255887ff5a09adbbd49f87a461799c010aea102c31335d65</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3490,39 +3482,39 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.3275</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Aberdeen vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
           <t>Aberdeen</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Aberdeen vs Heart of Midlothian</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Aberdeen</t>
-        </is>
-      </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>Heart of Midlothian</t>
@@ -3530,7 +3522,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3560,7 +3552,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1785598284</t>
+          <t>1785600627</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3570,7 +3562,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>3.053435</t>
+          <t>48.537549</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3587,7 +3579,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
+          <t>0x9928666cf9e1684bde5a3ebbe01a541c8265a2a2941c672ef774c0600b8a312d</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3595,31 +3587,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>37.20755</t>
+          <t>10.08</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.6025</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Aberdeen +0.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -3642,7 +3626,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3672,7 +3656,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1785598183</t>
+          <t>1785600583</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3682,7 +3666,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>62.797553</t>
+          <t>16.73029</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3699,7 +3683,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
+          <t>0xb5bac00ce7791648a87a47dcb5171aa144f49ab021c1a0dfad750f804d93836a</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3714,22 +3698,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>253.59</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.5925</t>
+          <t>1.3262</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Asian Handicap (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Aberdeen +0.5</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3754,7 +3738,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3784,7 +3768,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1785598181</t>
+          <t>1785600448</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3794,7 +3778,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>428.0</t>
+          <t>30.651341</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3811,7 +3795,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
+          <t>0x38706f9171542d01bce83eea0f508d61220ed3812837fd3378a4ba9378ad3044</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3819,28 +3803,36 @@
           <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>26.19</t>
+          <t>7.12</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.5437</t>
+          <t>1.3162</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>Aberdeen vs Heart of Midlothian</t>
@@ -3858,7 +3850,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
+          <t>0x04e9c93b2a3cdb04295c6e42b353a7f36caf0911c8f1d076ed9845d827b65319</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3888,7 +3880,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1785597811</t>
+          <t>1785600138</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3898,7 +3890,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>48.165517</t>
+          <t>22.513834</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3915,67 +3907,59 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
+          <t>0x0abfa4d97fa8b65021131d51b5e7a11807375335069de4074a6958eb5933bf1b</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>118.87998</t>
+          <t>622.70999</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.9175</t>
+          <t>1.5962</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Celtic</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Premiership</t>
-        </is>
-      </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Celtic vs Dundee FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Dundee FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19228045</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4000,17 +3984,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1785597330</t>
+          <t>1785599983</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1785781800</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>129.56946</t>
+          <t>1044.377342</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -4027,15 +4011,19 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
+          <t>0xf58dccabb95967ececb3018f2817565106376fd483b468b19405c12cb8a59ef0</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>0x7E3a6e22cac4eECeceCc7D9086d7c0fE1195Ec16</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>1</t>
@@ -4043,7 +4031,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.5837</t>
+          <t>1.3275</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4051,7 +4039,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Aberdeen</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4074,7 +4066,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
+          <t>0x62d76eb778a6607a159e32d82b64cfbf512384b97ecae550ec424b47239b43b6</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4104,7 +4096,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1785543200</t>
+          <t>1785598284</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4114,7 +4106,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>1.713062</t>
+          <t>3.053435</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4131,31 +4123,39 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
+          <t>0x9f0d5bbd68c46acf848124b165bc9e44a297569da9b235fd670f59e4806967f4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>40.29346</t>
+          <t>37.20755</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Aberdeen +0.5</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4163,27 +4163,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4208,17 +4208,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1785529916</t>
+          <t>1785598183</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>90.293468</t>
+          <t>62.797553</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4235,7 +4235,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
+          <t>0x32207acd736daa9a5552c759f251892aae7c67eae4995d245e53e2ae553b5041</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4243,23 +4243,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>253.59</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.4463</t>
+          <t>1.5925</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>Asian Handicap (0.5)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Aberdeen +0.5</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4267,27 +4275,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0xe279716d54dc617cd67bb4cb03a250c91fe3454ebf59dbcdeff34fb6943400c4</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4312,17 +4320,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1785529915</t>
+          <t>1785598181</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>2.577031</t>
+          <t>428.0</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4339,28 +4347,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
+          <t>0xf8991a6d899a35a1bbf1d6b29c0560594141a4c87048ff44daa3a7919d9b8b20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>26.19</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.4175</t>
+          <t>1.5437</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>Premiership</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
@@ -4371,27 +4379,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0xdea6c0813852afb4b4bf13cca885f2c863ecc81b5b718a5c2a162a3f0f1bb308</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4416,17 +4424,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1785529816</t>
+          <t>1785597811</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>2.754491</t>
+          <t>48.165517</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4443,31 +4451,39 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
+          <t>0xa84f14f5567e2b0ab922888be149003601a2966dcb690de037578a4f11fa4120</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+          <t>0x0fE55cE066A9810115Ea99B11a14e96a4b635810</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>118.87998</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.9175</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4475,27 +4491,27 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Celtic vs Dundee FC</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Dundee FC</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x1c5d0942acd8f3112cad4143a69702ae70fc03bc778aa6766837908f97e14fbf</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228045</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -4520,17 +4536,17 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1785529105</t>
+          <t>1785597330</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785781800</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>129.56946</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4547,7 +4563,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
+          <t>0xe833e969b88818e2354a4b8957b6d20896a41f4b0c3bb51d8ce17572c37d85b1</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4558,17 +4574,17 @@
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1.2612</t>
+          <t>1.5837</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
@@ -4579,27 +4595,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Dundee United vs Rangers FC</t>
+          <t>Aberdeen vs Heart of Midlothian</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Dundee United</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Rangers FC</t>
+          <t>Heart of Midlothian</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
+          <t>0x0744485ec0f21d4fce373018d4739c77bf4d61e274d73317a5bbfda23f87f48b</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>L19228047</t>
+          <t>L19228039</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4624,17 +4640,17 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785543200</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>1785524400</t>
+          <t>1785601800</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>6.77512</t>
+          <t>1.713062</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
@@ -4651,28 +4667,28 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
+          <t>0x38a2ec9c46673affecf2dd2e40bb35b3ce724ee1abcf2ea7bf46223f3d2dae29</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>40.29346</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -4698,7 +4714,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -4728,7 +4744,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>1785529104</t>
+          <t>1785529916</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -4738,7 +4754,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>1.587302</t>
+          <t>90.293468</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4755,39 +4771,31 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
+          <t>0x811525e57f52b3cd51b87498ca835dafe03edd882923f8b295bf84dba438dba9</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>75.44</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.1313</t>
+          <t>1.4463</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Under/Over (4.5)</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Over 4.5</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4810,7 +4818,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -4840,7 +4848,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785529915</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -4850,7 +4858,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>574.780952</t>
+          <t>2.577031</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -4867,39 +4875,31 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
+          <t>0x756c0d9d6c86ffc6c9a574910bef44e4e7a8572808cc31e7a38fe7d763b5bb12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>169.77</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.4175</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Under/Over (4)</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Over 4.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>1785526843</t>
+          <t>1785529816</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>1061.0625</t>
+          <t>2.754491</t>
         </is>
       </c>
       <c r="U42" t="inlineStr">
@@ -4979,7 +4979,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+          <t>0x9190b7571f2e54f6eeb0960c36b8e7815945cd0272019485a9ed234a596e5e0c</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4990,17 +4990,17 @@
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>20.18</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>1.3887</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5056,7 +5056,7 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>1785526560</t>
+          <t>1785529105</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>51.909968</t>
+          <t>1.587302</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5083,39 +5083,31 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+          <t>0x9f8081a9f8d3cf12a4a6ef88f2c8a5b07d8d8deb1bf4e72aeadad4553f251e99</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>61.03</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1.0925</t>
+          <t>1.2612</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Under/Over (5)</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Over 5.0</t>
-        </is>
-      </c>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>Premiership</t>
@@ -5138,7 +5130,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+          <t>0x134066d0292ae65674d11acfc245189b0f5932f143c0a3f1508a373a813e3370</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -5168,7 +5160,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>1785524635</t>
+          <t>1785529104</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -5178,7 +5170,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>659.783784</t>
+          <t>6.77512</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5195,110 +5187,654 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>0x7823d9cbc25df4d2ce923f58fdd31cdf09205f13511bea821d348907cd22f22b</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0xf4790f2265dea909876b7e0ddbb9612ac90d7a9e27eb0f3a900718ee6f3d4d8d</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1785529104</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>1.587302</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0x8eab29b3cce3f4590878b635836cd9dfe77938580dd4c4e944609e2f28faee9f</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>75.44</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.1313</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Under/Over (4.5)</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Over 4.5</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0x8ce8caee1fc33396cbda0b25dd4e673601e00cb200433d43cbc7ba6557ab6a27</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1785526843</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>574.780952</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0x75093cdd72db1ee3eae26e5ff6b6b750f8c641928612fa8fc050e56e073b27cf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>169.77</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Under/Over (4)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Over 4.0</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0xaef8117e7be3102f22003e6f0ba8d793562daea0942b2a11fa4604e29487dabf</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1785526843</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>1061.0625</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0x512f75a4e040002ce3fcaac79c15ee564e7d883b0c6f03de771b74316f733540</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>20.18</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.3887</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0xe1678df7687688d2ba9549ce444adeb9cc47cb904df706528a6fe7b9800dc519</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1785526560</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>51.909968</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0x1c754a278d7506d77f69973cf1876693bd5c2beb11810930bf32075703a0f973</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0x8268feC8dCb0D284343054BDf2b649286c9aA0a1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>61.03</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.0925</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Under/Over (5)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Over 5.0</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Premiership</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Dundee United vs Rangers FC</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Dundee United</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Rangers FC</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0x754c07be0249040cb3ac1bfbc49ca63bd34d58e9cfc2ec300ae5eab844f3a05b</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19228047</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1785524635</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1785524400</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>659.783784</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>0x3a6afc0d74597a50f894e10c8d93084fcb7ca5e09aa24a3eab1b5f521c2b6e08</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>0xCCdf6F3306aa9df4a4852FaF67fA1e1D58c4Db4e</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
         <is>
           <t>176.04</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>1.495</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Under/Over (3)</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>Over 3.0</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>Premiership</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Dundee United vs Rangers FC</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>Dundee United</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Rangers FC</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>0x2af09a7c30a9c2f3a49f480d1eba3b8573b203b8cb5cec998c89bf8da583850a</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>L19228047</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
         <is>
           <t>1785524138</t>
         </is>
       </c>
-      <c r="S45" t="inlineStr">
+      <c r="S50" t="inlineStr">
         <is>
           <t>1785524400</t>
         </is>
       </c>
-      <c r="T45" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>355.636364</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
+      <c r="V50" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>